<commit_message>
Borde de botones mas grueso
Borde de botones mas grueso
</commit_message>
<xml_diff>
--- a/Circuito/dom32-touch-Materiales.xlsx
+++ b/Circuito/dom32-touch-Materiales.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2708d86aa79f336/Documentos/Git/dom32-touch/Circuito/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="8_{AB4AD6D3-1ADD-4753-B268-0A87D7AF4A59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5030820C-44E4-4EBF-A19D-C07317CACCAD}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="8_{AB4AD6D3-1ADD-4753-B268-0A87D7AF4A59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{714310BF-C0C7-45BB-A7C7-31534E157476}"/>
   <bookViews>
-    <workbookView xWindow="11430" yWindow="1755" windowWidth="20910" windowHeight="12660" xr2:uid="{954617B2-1595-4720-8356-B08278AFF7FB}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{954617B2-1595-4720-8356-B08278AFF7FB}"/>
   </bookViews>
   <sheets>
     <sheet name="dom32-touch-Materiales" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
   <si>
     <t>Identificador</t>
   </si>
@@ -164,6 +164,15 @@
   </si>
   <si>
     <t>PIC32MM0256GPM028-I-SS</t>
+  </si>
+  <si>
+    <t>Display</t>
+  </si>
+  <si>
+    <t>AFY240320B0-2.4N6NTM-R</t>
+  </si>
+  <si>
+    <t>https://www.orientdisplay.com/products/afy240320b0-2-4n6ntm-r-2-4-tft-370-nits/</t>
   </si>
 </sst>
 </file>
@@ -1024,15 +1033,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A16E2AA9-FDD7-43B1-89C6-37BF40832499}">
-  <dimension ref="A1:C23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="42.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="42.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="30" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1043,7 +1052,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -1054,7 +1063,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -1065,7 +1074,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -1076,7 +1085,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1087,7 +1096,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>39</v>
       </c>
@@ -1098,7 +1107,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -1109,7 +1118,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -1120,7 +1129,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -1131,7 +1140,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>35</v>
       </c>
@@ -1142,7 +1151,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>43</v>
       </c>
@@ -1153,7 +1162,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>5</v>
       </c>
@@ -1164,7 +1173,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>15</v>
       </c>
@@ -1175,7 +1184,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>37</v>
       </c>
@@ -1186,7 +1195,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>7</v>
       </c>
@@ -1197,7 +1206,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>17</v>
       </c>
@@ -1208,7 +1217,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>23</v>
       </c>
@@ -1219,7 +1228,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>9</v>
       </c>
@@ -1230,7 +1239,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>27</v>
       </c>
@@ -1241,7 +1250,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>33</v>
       </c>
@@ -1252,7 +1261,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>31</v>
       </c>
@@ -1263,7 +1272,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>45</v>
       </c>
@@ -1274,7 +1283,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>41</v>
       </c>
@@ -1283,6 +1292,20 @@
       </c>
       <c r="C23" t="s">
         <v>42</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>47</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>48</v>
+      </c>
+      <c r="D24" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>